<commit_message>
special comment task added
</commit_message>
<xml_diff>
--- a/data/bulk_special_task_creation_valid.xlsx
+++ b/data/bulk_special_task_creation_valid.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t>Task Name*</t>
   </si>
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
@@ -687,15 +687,66 @@
         <v>38</v>
       </c>
       <c r="B3" s="3">
-        <v>46211</v>
+        <v>46226</v>
       </c>
       <c r="C3" s="3">
-        <v>46211</v>
+        <v>46226</v>
       </c>
       <c r="K3" t="s">
         <v>36</v>
       </c>
       <c r="P3" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" s="1" customFormat="1">
+      <c r="A4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46226</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46226</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" s="1" customFormat="1">
+      <c r="A5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46226</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46226</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" s="1" customFormat="1">
+      <c r="A6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46226</v>
+      </c>
+      <c r="C6" s="3">
+        <v>46226</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>